<commit_message>
Add cloud quotation API backed by Excel Master_DB
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel-quote/WAC_Air_Quotation_Simulator.xlsx
+++ b/excel-quote/WAC_Air_Quotation_Simulator.xlsx
@@ -2705,7 +2705,7 @@
         <f>IFERROR((IF(J18="",I18,J18)+IF(J19="",I19,J19)+IF(J20="",I20,J20)+IF(J21="",I21,J21)+IF(J22="",I22,J22)+IF(J23="",I23,J23)+IF(J24="",I24,J24)+IF(J25="",I25,J25)+IF(J26="",I26,J26)+IF(J27="",I27,J27)+IF(J28="",I28,J28)+IF(J29="",I29,J29)+IF(J30="",I30,J30))*IF(C33="HKD",C34,1),"")</f>
         <v/>
       </c>
-      <c r="J31" s="90" t="n"/>
+      <c r="J31" s="85" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="34" t="n"/>
@@ -2715,8 +2715,8 @@
       <c r="F32" s="92" t="n"/>
       <c r="G32" s="92" t="n"/>
       <c r="H32" s="93" t="n"/>
-      <c r="I32" s="91" t="n"/>
-      <c r="J32" s="93" t="n"/>
+      <c r="I32" s="86" t="n"/>
+      <c r="J32" s="87" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="43" t="inlineStr">
@@ -3438,7 +3438,7 @@
         <f>IFERROR(IF(입력!J18="",입력!I18,입력!J18)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G26" s="66" t="n"/>
+      <c r="G26" s="106" t="n"/>
     </row>
     <row r="27" ht="19.95" customHeight="1" s="62">
       <c r="B27" s="108">
@@ -3452,7 +3452,7 @@
         <f>IFERROR(IF(입력!J19="",입력!I19,입력!J19)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G27" s="66" t="n"/>
+      <c r="G27" s="106" t="n"/>
     </row>
     <row r="28" ht="31.95" customHeight="1" s="62">
       <c r="B28" s="108">
@@ -3466,7 +3466,7 @@
         <f>IFERROR(IF(입력!J20="",입력!I20,입력!J20)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G28" s="66" t="n"/>
+      <c r="G28" s="106" t="n"/>
     </row>
     <row r="29" ht="19.95" customHeight="1" s="62">
       <c r="B29" s="108">
@@ -3480,7 +3480,7 @@
         <f>IFERROR(IF(입력!J21="",입력!I21,입력!J21)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G29" s="66" t="n"/>
+      <c r="G29" s="106" t="n"/>
     </row>
     <row r="30" ht="19.95" customHeight="1" s="62">
       <c r="B30" s="108">
@@ -3494,7 +3494,7 @@
         <f>IFERROR(IF(입력!J22="",입력!I22,입력!J22)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G30" s="66" t="n"/>
+      <c r="G30" s="106" t="n"/>
     </row>
     <row r="31" ht="19.95" customHeight="1" s="62">
       <c r="B31" s="108">
@@ -3508,7 +3508,7 @@
         <f>IFERROR(IF(입력!J23="",입력!I23,입력!J23)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G31" s="66" t="n"/>
+      <c r="G31" s="106" t="n"/>
     </row>
     <row r="32" ht="19.95" customHeight="1" s="62">
       <c r="B32" s="108">
@@ -3522,7 +3522,7 @@
         <f>IFERROR(IF(입력!J24="",입력!I24,입력!J24)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G32" s="66" t="n"/>
+      <c r="G32" s="106" t="n"/>
     </row>
     <row r="33" ht="19.95" customHeight="1" s="62">
       <c r="B33" s="108">
@@ -3536,7 +3536,7 @@
         <f>IFERROR(IF(입력!J25="",입력!I25,입력!J25)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G33" s="66" t="n"/>
+      <c r="G33" s="106" t="n"/>
     </row>
     <row r="34" ht="19.95" customHeight="1" s="62">
       <c r="B34" s="108">
@@ -3550,7 +3550,7 @@
         <f>IFERROR(IF(입력!J26="",입력!I26,입력!J26)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G34" s="66" t="n"/>
+      <c r="G34" s="106" t="n"/>
     </row>
     <row r="35" ht="19.95" customHeight="1" s="62">
       <c r="B35" s="108">
@@ -3564,7 +3564,7 @@
         <f>IFERROR(IF(입력!J27="",입력!I27,입력!J27)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G35" s="66" t="n"/>
+      <c r="G35" s="106" t="n"/>
     </row>
     <row r="36" ht="19.95" customHeight="1" s="62">
       <c r="B36" s="108">
@@ -3578,7 +3578,7 @@
         <f>IFERROR(IF(입력!J28="",입력!I28,입력!J28)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G36" s="66" t="n"/>
+      <c r="G36" s="106" t="n"/>
     </row>
     <row r="37" ht="19.95" customHeight="1" s="62">
       <c r="B37" s="108">
@@ -3592,7 +3592,7 @@
         <f>IFERROR(IF(입력!J29="",입력!I29,입력!J29)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G37" s="66" t="n"/>
+      <c r="G37" s="106" t="n"/>
     </row>
     <row r="38" ht="19.95" customHeight="1" s="62">
       <c r="B38" s="108">
@@ -3606,7 +3606,7 @@
         <f>IFERROR(IF(입력!J30="",입력!I30,입력!J30)*IF(입력!C33="HKD",입력!C34,1),"")</f>
         <v/>
       </c>
-      <c r="G38" s="66" t="n"/>
+      <c r="G38" s="106" t="n"/>
     </row>
     <row r="39" ht="28" customHeight="1" s="62">
       <c r="B39" s="88" t="inlineStr">
@@ -3621,7 +3621,7 @@
         <f>입력!I31</f>
         <v/>
       </c>
-      <c r="G39" s="90" t="n"/>
+      <c r="G39" s="111" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1" s="62">
       <c r="B40" s="34" t="n"/>

</xml_diff>